<commit_message>
Cambio en la prueba F
</commit_message>
<xml_diff>
--- a/resultados_algoritmos/intervalos_confianza.xlsx
+++ b/resultados_algoritmos/intervalos_confianza.xlsx
@@ -471,19 +471,19 @@
         <v>100</v>
       </c>
       <c r="D2" t="n">
-        <v>0.1655408210353926</v>
+        <v>0.2729810003074817</v>
       </c>
       <c r="E2" t="n">
-        <v>0.01522256530057944</v>
+        <v>0.01924780380386367</v>
       </c>
       <c r="F2" t="n">
-        <v>1.984216951508683</v>
+        <v>1.984216951586417</v>
       </c>
       <c r="G2" t="n">
-        <v>0.1625203338239068</v>
+        <v>0.2691618184486382</v>
       </c>
       <c r="H2" t="n">
-        <v>0.1685613082468783</v>
+        <v>0.2768001821663253</v>
       </c>
     </row>
     <row r="3">
@@ -499,19 +499,19 @@
         <v>100</v>
       </c>
       <c r="D3" t="n">
-        <v>0.07274922973010689</v>
+        <v>0.1372599996102508</v>
       </c>
       <c r="E3" t="n">
-        <v>0.008869236792816598</v>
+        <v>0.01573240140555266</v>
       </c>
       <c r="F3" t="n">
-        <v>1.984216951508683</v>
+        <v>1.984216951586417</v>
       </c>
       <c r="G3" t="n">
-        <v>0.07098938073098177</v>
+        <v>0.1341383498544449</v>
       </c>
       <c r="H3" t="n">
-        <v>0.07450907872923201</v>
+        <v>0.1403816493660568</v>
       </c>
     </row>
     <row r="4">
@@ -527,19 +527,19 @@
         <v>100</v>
       </c>
       <c r="D4" t="n">
-        <v>0.0647045680670999</v>
+        <v>0.1014040001609828</v>
       </c>
       <c r="E4" t="n">
-        <v>0.006280875409744638</v>
+        <v>0.008710656640184692</v>
       </c>
       <c r="F4" t="n">
-        <v>1.984216951508683</v>
+        <v>1.984216951586417</v>
       </c>
       <c r="G4" t="n">
-        <v>0.06345830612126696</v>
+        <v>0.0996756169044925</v>
       </c>
       <c r="H4" t="n">
-        <v>0.06595083001293284</v>
+        <v>0.1031323834174732</v>
       </c>
     </row>
     <row r="5">
@@ -555,19 +555,19 @@
         <v>100</v>
       </c>
       <c r="D5" t="n">
-        <v>1.023375431250315</v>
+        <v>1.698840000026394</v>
       </c>
       <c r="E5" t="n">
-        <v>0.05185582354199015</v>
+        <v>0.07273575697665392</v>
       </c>
       <c r="F5" t="n">
-        <v>1.984216951508683</v>
+        <v>1.984216951586417</v>
       </c>
       <c r="G5" t="n">
-        <v>1.013086110839669</v>
+        <v>1.684407647828439</v>
       </c>
       <c r="H5" t="n">
-        <v>1.033664751660961</v>
+        <v>1.713272352224348</v>
       </c>
     </row>
     <row r="6">
@@ -583,19 +583,19 @@
         <v>100</v>
       </c>
       <c r="D6" t="n">
-        <v>0.4372382900328375</v>
+        <v>0.8268449992465321</v>
       </c>
       <c r="E6" t="n">
-        <v>0.08171393614303485</v>
+        <v>0.06755634654890917</v>
       </c>
       <c r="F6" t="n">
-        <v>1.984216951508683</v>
+        <v>1.984216951586417</v>
       </c>
       <c r="G6" t="n">
-        <v>0.4210244723058867</v>
+        <v>0.8134403544455728</v>
       </c>
       <c r="H6" t="n">
-        <v>0.4534521077597883</v>
+        <v>0.8402496440474914</v>
       </c>
     </row>
     <row r="7">
@@ -611,19 +611,19 @@
         <v>100</v>
       </c>
       <c r="D7" t="n">
-        <v>0.1786537872976623</v>
+        <v>0.2750829995784443</v>
       </c>
       <c r="E7" t="n">
-        <v>0.03138082388768467</v>
+        <v>0.009046714416341955</v>
       </c>
       <c r="F7" t="n">
-        <v>1.984216951508683</v>
+        <v>1.984216951586417</v>
       </c>
       <c r="G7" t="n">
-        <v>0.1724271510266371</v>
+        <v>0.2732879351683376</v>
       </c>
       <c r="H7" t="n">
-        <v>0.1848804235686876</v>
+        <v>0.276878063988551</v>
       </c>
     </row>
     <row r="8">
@@ -639,19 +639,19 @@
         <v>100</v>
       </c>
       <c r="D8" t="n">
-        <v>4.690569540834986</v>
+        <v>7.16790599966771</v>
       </c>
       <c r="E8" t="n">
-        <v>0.1204403436467952</v>
+        <v>0.2111764565036592</v>
       </c>
       <c r="F8" t="n">
-        <v>1.984216951508683</v>
+        <v>1.984216951586417</v>
       </c>
       <c r="G8" t="n">
-        <v>4.666671563684035</v>
+        <v>7.126004009190659</v>
       </c>
       <c r="H8" t="n">
-        <v>4.714467517985936</v>
+        <v>7.20980799014476</v>
       </c>
     </row>
     <row r="9">
@@ -667,19 +667,19 @@
         <v>100</v>
       </c>
       <c r="D9" t="n">
-        <v>1.940785930491984</v>
+        <v>3.354983000317588</v>
       </c>
       <c r="E9" t="n">
-        <v>0.08692375153114092</v>
+        <v>0.151184763246915</v>
       </c>
       <c r="F9" t="n">
-        <v>1.984216951508683</v>
+        <v>1.984216951586417</v>
       </c>
       <c r="G9" t="n">
-        <v>1.923538372364302</v>
+        <v>3.324984663311978</v>
       </c>
       <c r="H9" t="n">
-        <v>1.958033488619666</v>
+        <v>3.384981337323199</v>
       </c>
     </row>
     <row r="10">
@@ -695,19 +695,19 @@
         <v>100</v>
       </c>
       <c r="D10" t="n">
-        <v>0.3770537310629152</v>
+        <v>0.5969109995930921</v>
       </c>
       <c r="E10" t="n">
-        <v>0.01697718995459087</v>
+        <v>0.02009982110220237</v>
       </c>
       <c r="F10" t="n">
-        <v>1.984216951508683</v>
+        <v>1.984216951586417</v>
       </c>
       <c r="G10" t="n">
-        <v>0.3736850882532269</v>
+        <v>0.5929227590176077</v>
       </c>
       <c r="H10" t="n">
-        <v>0.3804223738726034</v>
+        <v>0.6008992401685765</v>
       </c>
     </row>
     <row r="11">
@@ -723,19 +723,19 @@
         <v>100</v>
       </c>
       <c r="D11" t="n">
-        <v>21.61344541906146</v>
+        <v>30.79590399967856</v>
       </c>
       <c r="E11" t="n">
-        <v>0.5459495206220576</v>
+        <v>0.5902968383634838</v>
       </c>
       <c r="F11" t="n">
-        <v>1.984216951508683</v>
+        <v>1.984216951586417</v>
       </c>
       <c r="G11" t="n">
-        <v>21.50511718971283</v>
+        <v>30.67877630036369</v>
       </c>
       <c r="H11" t="n">
-        <v>21.7217736484101</v>
+        <v>30.91303169899343</v>
       </c>
     </row>
     <row r="12">
@@ -751,19 +751,19 @@
         <v>100</v>
       </c>
       <c r="D12" t="n">
-        <v>8.803667449974455</v>
+        <v>13.72096699968097</v>
       </c>
       <c r="E12" t="n">
-        <v>0.5545565430287969</v>
+        <v>0.3585306775826426</v>
       </c>
       <c r="F12" t="n">
-        <v>1.984216951508683</v>
+        <v>1.984216951586417</v>
       </c>
       <c r="G12" t="n">
-        <v>8.693631400649675</v>
+        <v>13.64982673486864</v>
       </c>
       <c r="H12" t="n">
-        <v>8.913703499299235</v>
+        <v>13.79210726449329</v>
       </c>
     </row>
     <row r="13">
@@ -779,19 +779,19 @@
         <v>100</v>
       </c>
       <c r="D13" t="n">
-        <v>0.8294829292572103</v>
+        <v>1.303662999998778</v>
       </c>
       <c r="E13" t="n">
-        <v>0.02837762304826024</v>
+        <v>0.09508254402876685</v>
       </c>
       <c r="F13" t="n">
-        <v>1.984216951508683</v>
+        <v>1.984216951586417</v>
       </c>
       <c r="G13" t="n">
-        <v>0.8238521931876222</v>
+        <v>1.284796560432594</v>
       </c>
       <c r="H13" t="n">
-        <v>0.8351136653267985</v>
+        <v>1.322529439564962</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Ultimos cambios y ajustes a los puntos
</commit_message>
<xml_diff>
--- a/resultados_algoritmos/intervalos_confianza.xlsx
+++ b/resultados_algoritmos/intervalos_confianza.xlsx
@@ -471,19 +471,19 @@
         <v>100</v>
       </c>
       <c r="D2" t="n">
-        <v>0.2729810003074817</v>
+        <v>0.1657866488676518</v>
       </c>
       <c r="E2" t="n">
-        <v>0.01924780380386367</v>
+        <v>0.01824228509334397</v>
       </c>
       <c r="F2" t="n">
-        <v>1.984216951586417</v>
+        <v>1.984216951508683</v>
       </c>
       <c r="G2" t="n">
-        <v>0.2691618184486382</v>
+        <v>0.1621669837360051</v>
       </c>
       <c r="H2" t="n">
-        <v>0.2768001821663253</v>
+        <v>0.1694063139992985</v>
       </c>
     </row>
     <row r="3">
@@ -499,19 +499,19 @@
         <v>100</v>
       </c>
       <c r="D3" t="n">
-        <v>0.1372599996102508</v>
+        <v>0.07137580832932144</v>
       </c>
       <c r="E3" t="n">
-        <v>0.01573240140555266</v>
+        <v>0.008418361783228502</v>
       </c>
       <c r="F3" t="n">
-        <v>1.984216951586417</v>
+        <v>1.984216951508683</v>
       </c>
       <c r="G3" t="n">
-        <v>0.1341383498544449</v>
+        <v>0.06970542271389996</v>
       </c>
       <c r="H3" t="n">
-        <v>0.1403816493660568</v>
+        <v>0.07304619394474293</v>
       </c>
     </row>
     <row r="4">
@@ -527,19 +527,19 @@
         <v>100</v>
       </c>
       <c r="D4" t="n">
-        <v>0.1014040001609828</v>
+        <v>0.06460836069891229</v>
       </c>
       <c r="E4" t="n">
-        <v>0.008710656640184692</v>
+        <v>0.009019213727103006</v>
       </c>
       <c r="F4" t="n">
-        <v>1.984216951586417</v>
+        <v>1.984216951508683</v>
       </c>
       <c r="G4" t="n">
-        <v>0.0996756169044925</v>
+        <v>0.06281875302225254</v>
       </c>
       <c r="H4" t="n">
-        <v>0.1031323834174732</v>
+        <v>0.06639796837557205</v>
       </c>
     </row>
     <row r="5">
@@ -555,19 +555,19 @@
         <v>100</v>
       </c>
       <c r="D5" t="n">
-        <v>1.698840000026394</v>
+        <v>1.030764170864131</v>
       </c>
       <c r="E5" t="n">
-        <v>0.07273575697665392</v>
+        <v>0.05608057751366875</v>
       </c>
       <c r="F5" t="n">
-        <v>1.984216951586417</v>
+        <v>1.984216951508683</v>
       </c>
       <c r="G5" t="n">
-        <v>1.684407647828439</v>
+        <v>1.019636567608829</v>
       </c>
       <c r="H5" t="n">
-        <v>1.713272352224348</v>
+        <v>1.041891774119433</v>
       </c>
     </row>
     <row r="6">
@@ -583,19 +583,19 @@
         <v>100</v>
       </c>
       <c r="D6" t="n">
-        <v>0.8268449992465321</v>
+        <v>0.4309103798004799</v>
       </c>
       <c r="E6" t="n">
-        <v>0.06755634654890917</v>
+        <v>0.03744400717447883</v>
       </c>
       <c r="F6" t="n">
-        <v>1.984216951586417</v>
+        <v>1.984216951508683</v>
       </c>
       <c r="G6" t="n">
-        <v>0.8134403544455728</v>
+        <v>0.4234806764236785</v>
       </c>
       <c r="H6" t="n">
-        <v>0.8402496440474914</v>
+        <v>0.4383400831772812</v>
       </c>
     </row>
     <row r="7">
@@ -611,19 +611,19 @@
         <v>100</v>
       </c>
       <c r="D7" t="n">
-        <v>0.2750829995784443</v>
+        <v>0.1752259107888676</v>
       </c>
       <c r="E7" t="n">
-        <v>0.009046714416341955</v>
+        <v>0.009034221634301908</v>
       </c>
       <c r="F7" t="n">
-        <v>1.984216951586417</v>
+        <v>1.984216951508683</v>
       </c>
       <c r="G7" t="n">
-        <v>0.2732879351683376</v>
+        <v>0.1734333252178208</v>
       </c>
       <c r="H7" t="n">
-        <v>0.276878063988551</v>
+        <v>0.1770184963599145</v>
       </c>
     </row>
     <row r="8">
@@ -639,19 +639,19 @@
         <v>100</v>
       </c>
       <c r="D8" t="n">
-        <v>7.16790599966771</v>
+        <v>4.732015437330119</v>
       </c>
       <c r="E8" t="n">
-        <v>0.2111764565036592</v>
+        <v>0.131007962750837</v>
       </c>
       <c r="F8" t="n">
-        <v>1.984216951586417</v>
+        <v>1.984216951508683</v>
       </c>
       <c r="G8" t="n">
-        <v>7.126004009190659</v>
+        <v>4.706020615282837</v>
       </c>
       <c r="H8" t="n">
-        <v>7.20980799014476</v>
+        <v>4.758010259377402</v>
       </c>
     </row>
     <row r="9">
@@ -667,19 +667,19 @@
         <v>100</v>
       </c>
       <c r="D9" t="n">
-        <v>3.354983000317588</v>
+        <v>1.995271278719883</v>
       </c>
       <c r="E9" t="n">
-        <v>0.151184763246915</v>
+        <v>0.4099461150868464</v>
       </c>
       <c r="F9" t="n">
-        <v>1.984216951586417</v>
+        <v>1.984216951508683</v>
       </c>
       <c r="G9" t="n">
-        <v>3.324984663311978</v>
+        <v>1.913929075643839</v>
       </c>
       <c r="H9" t="n">
-        <v>3.384981337323199</v>
+        <v>2.076613481795929</v>
       </c>
     </row>
     <row r="10">
@@ -695,19 +695,19 @@
         <v>100</v>
       </c>
       <c r="D10" t="n">
-        <v>0.5969109995930921</v>
+        <v>0.3837125009158626</v>
       </c>
       <c r="E10" t="n">
-        <v>0.02009982110220237</v>
+        <v>0.06088642789420749</v>
       </c>
       <c r="F10" t="n">
-        <v>1.984216951586417</v>
+        <v>1.984216951508683</v>
       </c>
       <c r="G10" t="n">
-        <v>0.5929227590176077</v>
+        <v>0.3716313126814129</v>
       </c>
       <c r="H10" t="n">
-        <v>0.6008992401685765</v>
+        <v>0.3957936891503124</v>
       </c>
     </row>
     <row r="11">
@@ -723,19 +723,19 @@
         <v>100</v>
       </c>
       <c r="D11" t="n">
-        <v>30.79590399967856</v>
+        <v>21.34521586063784</v>
       </c>
       <c r="E11" t="n">
-        <v>0.5902968383634838</v>
+        <v>0.2877965700064702</v>
       </c>
       <c r="F11" t="n">
-        <v>1.984216951586417</v>
+        <v>1.984216951508683</v>
       </c>
       <c r="G11" t="n">
-        <v>30.67877630036369</v>
+        <v>21.28811077735855</v>
       </c>
       <c r="H11" t="n">
-        <v>30.91303169899343</v>
+        <v>21.40232094391713</v>
       </c>
     </row>
     <row r="12">
@@ -751,19 +751,19 @@
         <v>100</v>
       </c>
       <c r="D12" t="n">
-        <v>13.72096699968097</v>
+        <v>8.672335450246464</v>
       </c>
       <c r="E12" t="n">
-        <v>0.3585306775826426</v>
+        <v>0.5387428218696483</v>
       </c>
       <c r="F12" t="n">
-        <v>1.984216951586417</v>
+        <v>1.984216951508683</v>
       </c>
       <c r="G12" t="n">
-        <v>13.64982673486864</v>
+        <v>8.565437186280727</v>
       </c>
       <c r="H12" t="n">
-        <v>13.79210726449329</v>
+        <v>8.779233714212202</v>
       </c>
     </row>
     <row r="13">
@@ -779,19 +779,19 @@
         <v>100</v>
       </c>
       <c r="D13" t="n">
-        <v>1.303662999998778</v>
+        <v>0.8174987803795375</v>
       </c>
       <c r="E13" t="n">
-        <v>0.09508254402876685</v>
+        <v>0.01658856030922527</v>
       </c>
       <c r="F13" t="n">
-        <v>1.984216951586417</v>
+        <v>1.984216951508683</v>
       </c>
       <c r="G13" t="n">
-        <v>1.284796560432594</v>
+        <v>0.8142072501228687</v>
       </c>
       <c r="H13" t="n">
-        <v>1.322529439564962</v>
+        <v>0.8207903106362063</v>
       </c>
     </row>
   </sheetData>

</xml_diff>